<commit_message>
feat(halavi): add family 908 סטנד equipment to reserve slots 61-81
21 display stands/equipment (pushers, rails, labels, stands) added to
halavi deep reserve בי 61-81 (מיקום 261-281).
Only appear in Excel מיקום output — not in expiry view (no batch data).

Fix: build-halavi-new.js cleaning logic now preserves breira-default
explicitly placed products (bdMakatSet check) so equipment stays through rebuilds.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planogram/breira-default/FOR-ALL.xlsx
+++ b/planogram/breira-default/FOR-ALL.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H212"/>
+  <dimension ref="A1:H233"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5911,9 +5911,555 @@
         <v>15</v>
       </c>
     </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B213">
+        <v>247</v>
+      </c>
+      <c r="C213">
+        <v>261</v>
+      </c>
+      <c r="D213">
+        <v>61</v>
+      </c>
+      <c r="E213">
+        <v>908001</v>
+      </c>
+      <c r="F213" t="str">
+        <v>(82X180) גדול צדדי דו סטנד</v>
+      </c>
+      <c r="G213" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H213" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B214">
+        <v>248</v>
+      </c>
+      <c r="C214">
+        <v>262</v>
+      </c>
+      <c r="D214">
+        <v>62</v>
+      </c>
+      <c r="E214">
+        <v>908002</v>
+      </c>
+      <c r="F214" t="str">
+        <v>(56X180) בינוני צדדי דו סטנד</v>
+      </c>
+      <c r="G214" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H214" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B215">
+        <v>249</v>
+      </c>
+      <c r="C215">
+        <v>263</v>
+      </c>
+      <c r="D215">
+        <v>63</v>
+      </c>
+      <c r="E215">
+        <v>908003</v>
+      </c>
+      <c r="F215" t="str">
+        <v>(50X168) קיר רשת</v>
+      </c>
+      <c r="G215" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H215" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B216">
+        <v>250</v>
+      </c>
+      <c r="C216">
+        <v>264</v>
+      </c>
+      <c r="D216">
+        <v>64</v>
+      </c>
+      <c r="E216">
+        <v>908004</v>
+      </c>
+      <c r="F216" t="str">
+        <v>'סמ20 לרשת וו</v>
+      </c>
+      <c r="G216" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H216" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B217">
+        <v>251</v>
+      </c>
+      <c r="C217">
+        <v>265</v>
+      </c>
+      <c r="D217">
+        <v>65</v>
+      </c>
+      <c r="E217">
+        <v>908005</v>
+      </c>
+      <c r="F217" t="str">
+        <v>(50X190) רשת סטנד</v>
+      </c>
+      <c r="G217" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H217" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B218">
+        <v>252</v>
+      </c>
+      <c r="C218">
+        <v>266</v>
+      </c>
+      <c r="D218">
+        <v>66</v>
+      </c>
+      <c r="E218">
+        <v>908006</v>
+      </c>
+      <c r="F218" t="str">
+        <v>'סמ30 לרשת וו</v>
+      </c>
+      <c r="G218" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H218" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B219">
+        <v>253</v>
+      </c>
+      <c r="C219">
+        <v>267</v>
+      </c>
+      <c r="D219">
+        <v>67</v>
+      </c>
+      <c r="E219">
+        <v>908007</v>
+      </c>
+      <c r="F219" t="str">
+        <v>NORD PORT לוגו 12.5 מגשית</v>
+      </c>
+      <c r="G219" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H219" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B220">
+        <v>254</v>
+      </c>
+      <c r="C220">
+        <v>268</v>
+      </c>
+      <c r="D220">
+        <v>68</v>
+      </c>
+      <c r="E220">
+        <v>908008</v>
+      </c>
+      <c r="F220" t="str">
+        <v>SANTA BREMOR לוגו 12.5 מגשית</v>
+      </c>
+      <c r="G220" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H220" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B221">
+        <v>255</v>
+      </c>
+      <c r="C221">
+        <v>269</v>
+      </c>
+      <c r="D221">
+        <v>69</v>
+      </c>
+      <c r="E221">
+        <v>908010</v>
+      </c>
+      <c r="F221" t="str">
+        <v>(55) 33X39X16.5 קירור צידנית</v>
+      </c>
+      <c r="G221" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H221" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B222">
+        <v>256</v>
+      </c>
+      <c r="C222">
+        <v>270</v>
+      </c>
+      <c r="D222">
+        <v>70</v>
+      </c>
+      <c r="E222">
+        <v>908011</v>
+      </c>
+      <c r="F222" t="str">
+        <v>DADU ('יח 5) 'ג250-325 קרימוש גלידות צידנית</v>
+      </c>
+      <c r="G222" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H222" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B223">
+        <v>257</v>
+      </c>
+      <c r="C223">
+        <v>271</v>
+      </c>
+      <c r="D223">
+        <v>71</v>
+      </c>
+      <c r="E223">
+        <v>908012</v>
+      </c>
+      <c r="F223" t="str">
+        <v>(100) הונגרית קוביה</v>
+      </c>
+      <c r="G223" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H223" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B224">
+        <v>258</v>
+      </c>
+      <c r="C224">
+        <v>272</v>
+      </c>
+      <c r="D224">
+        <v>72</v>
+      </c>
+      <c r="E224">
+        <v>908013</v>
+      </c>
+      <c r="F224" t="str">
+        <v>מגנטים 8 כולל מ"ס205X66 למקרר כיסוי</v>
+      </c>
+      <c r="G224" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H224" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B225">
+        <v>259</v>
+      </c>
+      <c r="C225">
+        <v>273</v>
+      </c>
+      <c r="D225">
+        <v>73</v>
+      </c>
+      <c r="E225">
+        <v>908014</v>
+      </c>
+      <c r="F225" t="str">
+        <v>סטריפ</v>
+      </c>
+      <c r="G225" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H225" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B226">
+        <v>260</v>
+      </c>
+      <c r="C226">
+        <v>274</v>
+      </c>
+      <c r="D226">
+        <v>74</v>
+      </c>
+      <c r="E226">
+        <v>908015</v>
+      </c>
+      <c r="F226" t="str">
+        <v>מקודד</v>
+      </c>
+      <c r="G226" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H226" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B227">
+        <v>261</v>
+      </c>
+      <c r="C227">
+        <v>275</v>
+      </c>
+      <c r="D227">
+        <v>75</v>
+      </c>
+      <c r="E227">
+        <v>908016</v>
+      </c>
+      <c r="F227" t="str">
+        <v>(50) ברמור סנטה לבנה צידנית</v>
+      </c>
+      <c r="G227" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H227" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B228">
+        <v>262</v>
+      </c>
+      <c r="C228">
+        <v>276</v>
+      </c>
+      <c r="D228">
+        <v>76</v>
+      </c>
+      <c r="E228">
+        <v>908017</v>
+      </c>
+      <c r="F228" t="str">
+        <v>(50) פורט נורד לבנה צידנית</v>
+      </c>
+      <c r="G228" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H228" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B229">
+        <v>263</v>
+      </c>
+      <c r="C229">
+        <v>277</v>
+      </c>
+      <c r="D229">
+        <v>77</v>
+      </c>
+      <c r="E229">
+        <v>908018</v>
+      </c>
+      <c r="F229" t="str">
+        <v>(50) קרימוש לבנה צידנית</v>
+      </c>
+      <c r="G229" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H229" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B230">
+        <v>264</v>
+      </c>
+      <c r="C230">
+        <v>278</v>
+      </c>
+      <c r="D230">
+        <v>78</v>
+      </c>
+      <c r="E230">
+        <v>908032</v>
+      </c>
+      <c r="F230" t="str">
+        <v>PUSHER NORD PORT דחפן</v>
+      </c>
+      <c r="G230" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H230" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B231">
+        <v>265</v>
+      </c>
+      <c r="C231">
+        <v>279</v>
+      </c>
+      <c r="D231">
+        <v>79</v>
+      </c>
+      <c r="E231">
+        <v>908033</v>
+      </c>
+      <c r="F231" t="str">
+        <v>PUSHER MATIES דחפן</v>
+      </c>
+      <c r="G231" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H231" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B232">
+        <v>266</v>
+      </c>
+      <c r="C232">
+        <v>280</v>
+      </c>
+      <c r="D232">
+        <v>80</v>
+      </c>
+      <c r="E232">
+        <v>908034</v>
+      </c>
+      <c r="F232" t="str">
+        <v>RELS מ"ס 90 מסילה</v>
+      </c>
+      <c r="G232" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H232" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>חלבי</v>
+      </c>
+      <c r="B233">
+        <v>267</v>
+      </c>
+      <c r="C233">
+        <v>281</v>
+      </c>
+      <c r="D233">
+        <v>81</v>
+      </c>
+      <c r="E233">
+        <v>908035</v>
+      </c>
+      <c r="F233" t="str">
+        <v>PUSHER PRESIDENT דחפן</v>
+      </c>
+      <c r="G233" t="str">
+        <v>סטנד</v>
+      </c>
+      <c r="H233" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H212"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H233"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(halavi-908): set haluka=3 for all 908 סטנד products in breira-default
908 products had empty חלוקה column → haluka=null → sorted to end in Excel
Now haluka=3 (last חלבי group) → appear after PRESIDENT group, before קפוא
</commit_message>
<xml_diff>
--- a/planogram/breira-default/FOR-ALL.xlsx
+++ b/planogram/breira-default/FOR-ALL.xlsx
@@ -5933,8 +5933,8 @@
       <c r="G213" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H213" t="str">
-        <v/>
+      <c r="H213">
+        <v>3</v>
       </c>
     </row>
     <row r="214">
@@ -5959,8 +5959,8 @@
       <c r="G214" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H214" t="str">
-        <v/>
+      <c r="H214">
+        <v>3</v>
       </c>
     </row>
     <row r="215">
@@ -5985,8 +5985,8 @@
       <c r="G215" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H215" t="str">
-        <v/>
+      <c r="H215">
+        <v>3</v>
       </c>
     </row>
     <row r="216">
@@ -6011,8 +6011,8 @@
       <c r="G216" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H216" t="str">
-        <v/>
+      <c r="H216">
+        <v>3</v>
       </c>
     </row>
     <row r="217">
@@ -6037,8 +6037,8 @@
       <c r="G217" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H217" t="str">
-        <v/>
+      <c r="H217">
+        <v>3</v>
       </c>
     </row>
     <row r="218">
@@ -6063,8 +6063,8 @@
       <c r="G218" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H218" t="str">
-        <v/>
+      <c r="H218">
+        <v>3</v>
       </c>
     </row>
     <row r="219">
@@ -6089,8 +6089,8 @@
       <c r="G219" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H219" t="str">
-        <v/>
+      <c r="H219">
+        <v>3</v>
       </c>
     </row>
     <row r="220">
@@ -6115,8 +6115,8 @@
       <c r="G220" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H220" t="str">
-        <v/>
+      <c r="H220">
+        <v>3</v>
       </c>
     </row>
     <row r="221">
@@ -6141,8 +6141,8 @@
       <c r="G221" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H221" t="str">
-        <v/>
+      <c r="H221">
+        <v>3</v>
       </c>
     </row>
     <row r="222">
@@ -6167,8 +6167,8 @@
       <c r="G222" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H222" t="str">
-        <v/>
+      <c r="H222">
+        <v>3</v>
       </c>
     </row>
     <row r="223">
@@ -6193,8 +6193,8 @@
       <c r="G223" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H223" t="str">
-        <v/>
+      <c r="H223">
+        <v>3</v>
       </c>
     </row>
     <row r="224">
@@ -6219,8 +6219,8 @@
       <c r="G224" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H224" t="str">
-        <v/>
+      <c r="H224">
+        <v>3</v>
       </c>
     </row>
     <row r="225">
@@ -6245,8 +6245,8 @@
       <c r="G225" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H225" t="str">
-        <v/>
+      <c r="H225">
+        <v>3</v>
       </c>
     </row>
     <row r="226">
@@ -6271,8 +6271,8 @@
       <c r="G226" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H226" t="str">
-        <v/>
+      <c r="H226">
+        <v>3</v>
       </c>
     </row>
     <row r="227">
@@ -6297,8 +6297,8 @@
       <c r="G227" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H227" t="str">
-        <v/>
+      <c r="H227">
+        <v>3</v>
       </c>
     </row>
     <row r="228">
@@ -6323,8 +6323,8 @@
       <c r="G228" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H228" t="str">
-        <v/>
+      <c r="H228">
+        <v>3</v>
       </c>
     </row>
     <row r="229">
@@ -6349,8 +6349,8 @@
       <c r="G229" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H229" t="str">
-        <v/>
+      <c r="H229">
+        <v>3</v>
       </c>
     </row>
     <row r="230">
@@ -6375,8 +6375,8 @@
       <c r="G230" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H230" t="str">
-        <v/>
+      <c r="H230">
+        <v>3</v>
       </c>
     </row>
     <row r="231">
@@ -6401,8 +6401,8 @@
       <c r="G231" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H231" t="str">
-        <v/>
+      <c r="H231">
+        <v>3</v>
       </c>
     </row>
     <row r="232">
@@ -6427,8 +6427,8 @@
       <c r="G232" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H232" t="str">
-        <v/>
+      <c r="H232">
+        <v>3</v>
       </c>
     </row>
     <row r="233">
@@ -6453,8 +6453,8 @@
       <c r="G233" t="str">
         <v>סטנד</v>
       </c>
-      <c r="H233" t="str">
-        <v/>
+      <c r="H233">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>